<commit_message>
update: correct 2026-07-10 Daily Brief update with enriched metadata
- Added DCBM-122 (ZHANG Shuichang), DCBM-123 (LI Guoxin), DCBM-124 (SUN Jinsheng)
- All from Petroleum Exploration and Development Vol.53 No.3, 2026
- Fixed brief_parser: now parses Section 5 candidate details for richer prose
- Fixed workbook_update: corrected 精读摘要 (Col C now Chinese title, Col E structured summary, Col M star rating, Col N upgrade status)
- Fixed workbook_update: 总览统计 now updates metadata rows + year distribution
- Master: 121 -> 124 records, ID continuous, zero duplicates
- Protected dirs unmodified
</commit_message>
<xml_diff>
--- a/01_Increment/2026-07-10_daily_brief_update/Deep_CBM_increment_20260710.xlsx
+++ b/01_Increment/2026-07-10_daily_brief_update/Deep_CBM_increment_20260710.xlsx
@@ -143,25 +143,32 @@
     <t>煤层气与煤岩气</t>
   </si>
   <si>
-    <t>建立生成阶段与成因类型认识</t>
-  </si>
-  <si>
-    <t>综合地质与成因分析，具体方法待全文核验</t>
-  </si>
-  <si>
-    <t>建立煤岩气生成阶段和成因类型框架，细节待全文核验</t>
-  </si>
-  <si>
-    <t>统一不同深度煤系气成因认识</t>
-  </si>
-  <si>
-    <t>摘要未正常加载，定量信息待补</t>
-  </si>
-  <si>
-    <t>强相关，适合概念边界和生产机理讨论</t>
-  </si>
-  <si>
-    <t>引言；理论基础；讨论</t>
+    <t>该文聚焦中国煤岩气的生成阶段和成因类型，属于煤层气—深部煤岩气概念体系和成藏分类研究。其核心价值在于尝试从煤岩热演化、气体赋存状态、储层特征和生产表现等维度，对不同深度和不同演化阶段的煤系气资源进行统一认识。</t>
+  </si>
+  <si>
+    <t>官方英文页面当前能够稳定核验题名、作者、卷期、页码、DOI 和出版时间，但摘要正文未正常加载。因此本次不能可靠提取具体样品数量、实验流程和定量参数。根据题名和文章类型，可判断其主要采用综合地质分析和成因分类方法，但该判断仍需 Codex 或人工阅读全文确认。</t>
+  </si>
+  <si>
+    <t>当前只能确认文章建立或讨论了中国煤岩气生成阶段与成因类型框架。更具体的分类边界、赋存相态演化和判别指标必须以全文为准，不应仅依据题名扩展为正式结论。</t>
+  </si>
+  <si>
+    <t>可能的创新在于将浅层煤层气、深部煤岩气及相关煤系气类型置于统一演化框架下讨论</t>
+  </si>
+  <si>
+    <t>当前局限是官方网页摘要未正常显示，无法从公开页面核验具体分类数量、阈值和定量结论</t>
+  </si>
+  <si>
+    <t>该文对用户当前先导井研究的直接数据贡献有限，但对以下内容高度相关：
+深部煤层气与煤岩气概念边界；
+深度增加后吸附气、游离气赋存关系变化；
+不同类型气藏生产机制差异；
+论文引言、理论基础和讨论章节的术语统一。</t>
+  </si>
+  <si>
+    <t>引言与研究背景；
+深部煤层气/煤岩气概念与成藏类型；
+排采响应差异的地质机理讨论；
+开发模式与生产机制讨论。</t>
   </si>
   <si>
     <t>煤岩气；生成阶段；成因类型；赋存状态</t>
@@ -203,25 +210,32 @@
     <t>煤岩气聚集过渡带</t>
   </si>
   <si>
-    <t>解释聚集过渡带形成机制</t>
-  </si>
-  <si>
-    <t>地质综合分析，具体方法待全文核验</t>
-  </si>
-  <si>
-    <t>提出聚集过渡带形成机制，具体控制因素待全文核验</t>
-  </si>
-  <si>
-    <t>将过渡带作为独立成藏评价对象</t>
-  </si>
-  <si>
-    <t>摘要未正常加载，研究区和定量数据待补</t>
-  </si>
-  <si>
-    <t>强相关，可支持井间响应差异的区域地质解释</t>
-  </si>
-  <si>
-    <t>区域地质；富集规律；讨论</t>
+    <t>该文研究煤岩气聚集过渡带的形成机制，重点应涉及煤岩气在区域成藏体系中的空间过渡、气体富集差异和地质边界特征。</t>
+  </si>
+  <si>
+    <t>官方页面能够稳定核验题名、作者、卷期、页码、DOI 和出版日期，但摘要内容未正常加载。当前无法确认研究区、样品量、测井资料、地球化学数据或数值模拟方法。Codex 入库时应从 PDF 或正式中文页面补齐这些字段。</t>
+  </si>
+  <si>
+    <t>根据题名可确认文章提出或解释了煤岩气聚集过渡带的形成机制，但具体机制组成、控制因素和区域适用性尚不能从当前公开页面可靠提取。</t>
+  </si>
+  <si>
+    <t>潜在创新是将“聚集过渡带”作为煤岩气成藏和有利区评价的独立对象</t>
+  </si>
+  <si>
+    <t>局限是当前摘要不可用，不能据此写入定量阈值、甜点范围或主控因素排序</t>
+  </si>
+  <si>
+    <t>该文可作为解释先导井之间响应差异的区域地质背景文献，尤其适用于：
+区块内富集带与过渡带划分；
+井间含气性和储层品质差异解释；
+响应类型与区域成藏位置之间的联系；
+有利区和开发单元划分的理论支持。</t>
+  </si>
+  <si>
+    <t>区域地质背景；
+煤岩气富集规律；
+井间生产响应差异讨论；
+地质—工程一体化评价。</t>
   </si>
   <si>
     <t>煤岩气；聚集过渡带；富集机制</t>
@@ -257,25 +271,28 @@
     <t>深层煤岩气长水平井</t>
   </si>
   <si>
-    <t>提升井壁稳定和孔裂隙封堵能力</t>
-  </si>
-  <si>
-    <t>钻井液体系研发与现场验证，具体参数待全文核验</t>
-  </si>
-  <si>
-    <t>形成胶结成膜固壁疏水钻井液技术</t>
-  </si>
-  <si>
-    <t>多机制耦合的井壁稳定体系</t>
+    <t>该文面向深层煤岩气长水平井钻井过程中的井壁稳定、孔裂隙封堵和流体侵入控制问题，属于钻完井工程技术研究。</t>
+  </si>
+  <si>
+    <t>题名表明其技术路线包括胶结、成膜、固壁和疏水控制。官方页面未正常展示摘要，当前无法核验钻井液配方、实验温压条件、岩样类型、现场井数和性能提升幅度。</t>
+  </si>
+  <si>
+    <t>能够确认文章提出并验证了一套适用于深层煤岩气长水平井的胶结成膜固壁疏水钻井液技术。任何关于封堵率、膨胀抑制率、井径扩大率或现场提速幅度的数字均需阅读全文后再写入。</t>
+  </si>
+  <si>
+    <t>潜在创新是将孔裂隙封堵、胶结成膜、井壁强化和疏水抑制组合到同一钻井液体系中</t>
   </si>
   <si>
     <t>与排采动态间接相关；定量结果待补</t>
   </si>
   <si>
-    <t>工程背景和井筒质量影响因素参考</t>
-  </si>
-  <si>
-    <t>工程背景；讨论</t>
+    <t>该文可用于解释钻完井质量对后续压裂、排液、井筒完整性和生产稳定性的潜在影响，但不宜直接用于排采动态分型或产能主控因素排序。</t>
+  </si>
+  <si>
+    <t>深部煤岩气工程技术背景；
+水平井钻完井难点；
+地质—工程影响因素讨论；
+研究局限与工程资料缺失说明。</t>
   </si>
   <si>
     <t>深层煤岩气；水平井；钻井液；井壁稳定</t>

</xml_diff>